<commit_message>
Now handling mixed-gender X 4x400 event with one C&C record
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96D7E93-B2F1-40A9-8DD2-4E3BC4F35429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E50BCB8-62A4-47C8-8638-67FC9DA13119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1130" yWindow="300" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="225">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -687,6 +687,33 @@
   </si>
   <si>
     <t>100HW</t>
+  </si>
+  <si>
+    <t>3:47.84</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/2b5d0366-516f-4e27-a5c4-99c75ab33f72</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Stu Dunlop email</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/6bdfd2a7-208d-4666-9b65-f70ef559bf27</t>
+  </si>
+  <si>
+    <t>Cambridge &amp; Coleridge Mixed Senior Team</t>
+  </si>
+  <si>
+    <t>8 Aug 2026</t>
+  </si>
+  <si>
+    <t>Hemel Hempstead</t>
+  </si>
+  <si>
+    <t>4x400</t>
   </si>
 </sst>
 </file>
@@ -1453,22 +1480,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
   <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
-    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.08984375" style="1"/>
+    <col min="2" max="3" width="17.3828125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.69140625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.3828125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="30.4609375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.07421875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -1501,7 +1528,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1531,7 +1558,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1563,7 +1590,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1589,7 +1616,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1615,7 +1642,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1641,7 +1668,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>47</v>
       </c>
@@ -1667,7 +1694,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1693,7 +1720,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1719,7 +1746,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>61</v>
       </c>
@@ -1745,7 +1772,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1771,7 +1798,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
@@ -1797,7 +1824,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>73</v>
       </c>
@@ -1823,7 +1850,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
@@ -1852,7 +1879,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
@@ -1881,7 +1908,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1910,7 +1937,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
@@ -1939,7 +1966,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>103</v>
       </c>
@@ -1965,7 +1992,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>111</v>
       </c>
@@ -1997,7 +2024,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>116</v>
       </c>
@@ -2029,7 +2056,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>123</v>
       </c>
@@ -2058,7 +2085,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>128</v>
       </c>
@@ -2087,7 +2114,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>129</v>
       </c>
@@ -2116,7 +2143,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>130</v>
       </c>
@@ -2145,7 +2172,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
         <v>137</v>
       </c>
@@ -2177,7 +2204,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
         <v>145</v>
       </c>
@@ -2209,7 +2236,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
         <v>148</v>
       </c>
@@ -2241,7 +2268,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
         <v>152</v>
       </c>
@@ -2273,7 +2300,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
         <v>154</v>
       </c>
@@ -2305,7 +2332,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="1" t="s">
         <v>155</v>
@@ -2338,7 +2365,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
         <v>159</v>
       </c>
@@ -2370,7 +2397,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
         <v>157</v>
       </c>
@@ -2402,7 +2429,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
         <v>161</v>
       </c>
@@ -2434,7 +2461,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
         <v>177</v>
       </c>
@@ -2466,7 +2493,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
         <v>178</v>
       </c>
@@ -2498,7 +2525,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
         <v>179</v>
       </c>
@@ -2530,7 +2557,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
         <v>190</v>
       </c>
@@ -2562,7 +2589,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B40" s="1" t="s">
         <v>197</v>
       </c>
@@ -2594,7 +2621,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B41" s="1" t="s">
         <v>196</v>
       </c>
@@ -2626,7 +2653,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B42" s="1" t="s">
         <v>210</v>
       </c>
@@ -2658,7 +2685,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B43" s="1" t="s">
         <v>211</v>
       </c>
@@ -2690,7 +2717,39 @@
         <v>125</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B44" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -2717,8 +2776,10 @@
     <hyperlink ref="E27" r:id="rId18" xr:uid="{3394B413-0143-4554-8881-5A939C20DACD}"/>
     <hyperlink ref="H42" r:id="rId19" xr:uid="{0AFBFB3D-A621-49B6-9AED-DFB855EAF16A}"/>
     <hyperlink ref="H43" r:id="rId20" xr:uid="{1469BDE7-0674-474D-A6CE-8CD56D1EF9BC}"/>
+    <hyperlink ref="H44" r:id="rId21" xr:uid="{05BC432F-67F1-48FD-A8F2-ECEDD9EA27CD}"/>
+    <hyperlink ref="E44" r:id="rId22" xr:uid="{57BEC75D-58ED-4103-9440-441EF783670D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId21"/>
+  <drawing r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding DR MV45 HM & M performances this year so far
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\powerof10-tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E50BCB8-62A4-47C8-8638-67FC9DA13119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BFCD41-F5D0-4C84-BA09-4E058A4802CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="230">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -714,6 +714,21 @@
   </si>
   <si>
     <t>4x400</t>
+  </si>
+  <si>
+    <t>WhatsApp message, po10</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/79e25f45-4a62-4763-b13e-2e5d318b23d2</t>
+  </si>
+  <si>
+    <t>David Raimondo</t>
+  </si>
+  <si>
+    <t>74:15</t>
+  </si>
+  <si>
+    <t>2:39:21</t>
   </si>
 </sst>
 </file>
@@ -1480,22 +1495,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
   <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.3828125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.69140625" style="1" customWidth="1"/>
-    <col min="5" max="10" width="17.3828125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.4609375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.07421875" style="1"/>
+    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -1528,7 +1543,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1558,7 +1573,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1590,7 +1605,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1616,7 +1631,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1642,7 +1657,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1668,7 +1683,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>47</v>
       </c>
@@ -1694,7 +1709,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1720,7 +1735,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1746,7 +1761,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>61</v>
       </c>
@@ -1772,7 +1787,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1798,7 +1813,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
@@ -1824,7 +1839,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>73</v>
       </c>
@@ -1850,7 +1865,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
@@ -1879,7 +1894,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
@@ -1908,7 +1923,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1937,7 +1952,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
@@ -1966,7 +1981,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>103</v>
       </c>
@@ -1992,7 +2007,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>111</v>
       </c>
@@ -2024,7 +2039,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>116</v>
       </c>
@@ -2056,7 +2071,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>123</v>
       </c>
@@ -2085,7 +2100,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>128</v>
       </c>
@@ -2114,7 +2129,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>129</v>
       </c>
@@ -2143,7 +2158,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>130</v>
       </c>
@@ -2172,7 +2187,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>137</v>
       </c>
@@ -2204,7 +2219,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>145</v>
       </c>
@@ -2236,7 +2251,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>148</v>
       </c>
@@ -2268,7 +2283,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>152</v>
       </c>
@@ -2300,7 +2315,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>154</v>
       </c>
@@ -2332,7 +2347,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="1" t="s">
         <v>155</v>
@@ -2365,7 +2380,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>159</v>
       </c>
@@ -2397,7 +2412,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>157</v>
       </c>
@@ -2429,7 +2444,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>161</v>
       </c>
@@ -2461,7 +2476,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>177</v>
       </c>
@@ -2493,7 +2508,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>178</v>
       </c>
@@ -2525,7 +2540,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>179</v>
       </c>
@@ -2557,7 +2572,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
         <v>190</v>
       </c>
@@ -2589,7 +2604,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>197</v>
       </c>
@@ -2621,7 +2636,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
         <v>196</v>
       </c>
@@ -2653,7 +2668,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>210</v>
       </c>
@@ -2685,7 +2700,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>211</v>
       </c>
@@ -2717,7 +2732,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" s="1" t="s">
         <v>216</v>
       </c>
@@ -2749,7 +2764,71 @@
         <v>219</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B45" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B46" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -2778,8 +2857,11 @@
     <hyperlink ref="H43" r:id="rId20" xr:uid="{1469BDE7-0674-474D-A6CE-8CD56D1EF9BC}"/>
     <hyperlink ref="H44" r:id="rId21" xr:uid="{05BC432F-67F1-48FD-A8F2-ECEDD9EA27CD}"/>
     <hyperlink ref="E44" r:id="rId22" xr:uid="{57BEC75D-58ED-4103-9440-441EF783670D}"/>
+    <hyperlink ref="H45" r:id="rId23" xr:uid="{D0792C45-BAFC-4F52-B4F2-11A93885349C}"/>
+    <hyperlink ref="E45" r:id="rId24" xr:uid="{F585287C-F712-4CA3-8322-FAA7A87B31F9}"/>
+    <hyperlink ref="E46" r:id="rId25" xr:uid="{D866423A-05EA-40C3-915B-0EB5226D0FC9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId23"/>
+  <drawing r:id="rId26"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added WM Berlin Marathon record
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BFCD41-F5D0-4C84-BA09-4E058A4802CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A6906D-F554-40ED-AB18-7C7093D4EE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="237">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -729,6 +729,27 @@
   </si>
   <si>
     <t>2:39:21</t>
+  </si>
+  <si>
+    <t>27 Sep 2026</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/8e09dc52-512c-41ff-94c1-0eee6ce9bb5a</t>
+  </si>
+  <si>
+    <t>William Mycroft</t>
+  </si>
+  <si>
+    <t>2:14:24</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/4f794d7b-5678-495d-9ce4-54897704855b</t>
+  </si>
+  <si>
+    <t>Alerted by Sarah Abramson</t>
   </si>
 </sst>
 </file>
@@ -2828,6 +2849,38 @@
         <v>225</v>
       </c>
     </row>
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B47" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
     <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>0</v>
@@ -2860,8 +2913,10 @@
     <hyperlink ref="H45" r:id="rId23" xr:uid="{D0792C45-BAFC-4F52-B4F2-11A93885349C}"/>
     <hyperlink ref="E45" r:id="rId24" xr:uid="{F585287C-F712-4CA3-8322-FAA7A87B31F9}"/>
     <hyperlink ref="E46" r:id="rId25" xr:uid="{D866423A-05EA-40C3-915B-0EB5226D0FC9}"/>
+    <hyperlink ref="E47" r:id="rId26" xr:uid="{8FCF358B-643B-486C-93EF-263E08879F14}"/>
+    <hyperlink ref="H47" r:id="rId27" xr:uid="{3817F920-5A47-4FB2-8326-2F5A26A2E982}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId26"/>
+  <drawing r:id="rId28"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding MB 10M MV55 performance
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A6906D-F554-40ED-AB18-7C7093D4EE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4375462-A713-4E00-8AE0-AC8C22F66510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="244">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -750,6 +750,27 @@
   </si>
   <si>
     <t>Alerted by Sarah Abramson</t>
+  </si>
+  <si>
+    <t>61:20</t>
+  </si>
+  <si>
+    <t>11 Oct 2026</t>
+  </si>
+  <si>
+    <t>Michael Buchallet</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/6d56d665-12e2-40aa-981a-955baf7e318c</t>
+  </si>
+  <si>
+    <t>Tiptree</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/76c79dad-7e3a-4ecf-8b8c-7e7ba4a74d41</t>
+  </si>
+  <si>
+    <t>Email to records@cnc address</t>
   </si>
 </sst>
 </file>
@@ -1516,22 +1537,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
   <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
-    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.08984375" style="1"/>
+    <col min="2" max="3" width="17.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -1564,7 +1585,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1594,7 +1615,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1626,7 +1647,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1652,7 +1673,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1678,7 +1699,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1704,7 +1725,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>47</v>
       </c>
@@ -1730,7 +1751,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1756,7 +1777,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1782,7 +1803,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>61</v>
       </c>
@@ -1808,7 +1829,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1834,7 +1855,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
@@ -1860,7 +1881,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>73</v>
       </c>
@@ -1886,7 +1907,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
@@ -1915,7 +1936,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
@@ -1944,7 +1965,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1973,7 +1994,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
@@ -2002,7 +2023,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B20" s="1" t="s">
         <v>103</v>
       </c>
@@ -2028,7 +2049,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B21" s="1" t="s">
         <v>111</v>
       </c>
@@ -2060,7 +2081,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B22" s="1" t="s">
         <v>116</v>
       </c>
@@ -2092,7 +2113,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
         <v>123</v>
       </c>
@@ -2121,7 +2142,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
         <v>128</v>
       </c>
@@ -2150,7 +2171,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
         <v>129</v>
       </c>
@@ -2179,7 +2200,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
         <v>130</v>
       </c>
@@ -2208,7 +2229,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
         <v>137</v>
       </c>
@@ -2240,7 +2261,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28" s="1" t="s">
         <v>145</v>
       </c>
@@ -2272,7 +2293,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
         <v>148</v>
       </c>
@@ -2304,7 +2325,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
         <v>152</v>
       </c>
@@ -2336,7 +2357,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
         <v>154</v>
       </c>
@@ -2368,7 +2389,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="1" t="s">
         <v>155</v>
@@ -2401,7 +2422,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B33" s="1" t="s">
         <v>159</v>
       </c>
@@ -2433,7 +2454,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B34" s="1" t="s">
         <v>157</v>
       </c>
@@ -2465,7 +2486,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
         <v>161</v>
       </c>
@@ -2497,7 +2518,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B36" s="1" t="s">
         <v>177</v>
       </c>
@@ -2529,7 +2550,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
         <v>178</v>
       </c>
@@ -2561,7 +2582,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
         <v>179</v>
       </c>
@@ -2593,7 +2614,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B39" s="1" t="s">
         <v>190</v>
       </c>
@@ -2625,7 +2646,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B40" s="1" t="s">
         <v>197</v>
       </c>
@@ -2657,7 +2678,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B41" s="1" t="s">
         <v>196</v>
       </c>
@@ -2689,7 +2710,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B42" s="1" t="s">
         <v>210</v>
       </c>
@@ -2721,7 +2742,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B43" s="1" t="s">
         <v>211</v>
       </c>
@@ -2753,7 +2774,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B44" s="1" t="s">
         <v>216</v>
       </c>
@@ -2785,7 +2806,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B45" s="1" t="s">
         <v>228</v>
       </c>
@@ -2817,7 +2838,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
         <v>229</v>
       </c>
@@ -2849,7 +2870,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
         <v>234</v>
       </c>
@@ -2881,7 +2902,39 @@
         <v>236</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B48" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -2915,8 +2968,10 @@
     <hyperlink ref="E46" r:id="rId25" xr:uid="{D866423A-05EA-40C3-915B-0EB5226D0FC9}"/>
     <hyperlink ref="E47" r:id="rId26" xr:uid="{8FCF358B-643B-486C-93EF-263E08879F14}"/>
     <hyperlink ref="H47" r:id="rId27" xr:uid="{3817F920-5A47-4FB2-8326-2F5A26A2E982}"/>
+    <hyperlink ref="E48" r:id="rId28" xr:uid="{37F11BF0-1593-4719-AB2D-686310137F16}"/>
+    <hyperlink ref="H48" r:id="rId29" xr:uid="{D8D78CE1-8495-4754-AEC0-3BE32C7103AA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId28"/>
+  <drawing r:id="rId30"/>
 </worksheet>
 </file>
</xml_diff>